<commit_message>
bug-fix: fine-tuned error message rendering and content
</commit_message>
<xml_diff>
--- a/sample/13Apr-10May_26.xlsx
+++ b/sample/13Apr-10May_26.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12000"/>
+    <workbookView windowWidth="25600" windowHeight="12000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="13Aprto10May" sheetId="1" r:id="rId1"/>
@@ -251,6 +251,13 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -314,13 +321,6 @@
       <sz val="10"/>
       <name val="Verdana"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -758,6 +758,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -783,17 +794,6 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -1137,59 +1137,62 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1198,7 +1201,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1207,26 +1210,22 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1241,69 +1240,69 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
@@ -1655,1736 +1654,1736 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" spans="1:45">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="41"/>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
-      <c r="S1" s="42"/>
-      <c r="T1" s="56"/>
-      <c r="U1" s="57"/>
-      <c r="V1" s="41"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
-      <c r="AA1" s="8"/>
-      <c r="AB1" s="8"/>
-      <c r="AC1" s="64"/>
-      <c r="AD1" s="8"/>
-      <c r="AE1" s="8"/>
-      <c r="AF1" s="8"/>
-      <c r="AG1" s="41"/>
-      <c r="AH1" s="8"/>
-      <c r="AI1" s="8"/>
-      <c r="AJ1" s="8"/>
-      <c r="AK1" s="8"/>
-      <c r="AL1" s="8"/>
-      <c r="AM1" s="8"/>
-      <c r="AN1" s="8"/>
-      <c r="AO1" s="8"/>
-      <c r="AP1" s="8"/>
-      <c r="AQ1" s="8"/>
-      <c r="AR1" s="41"/>
-      <c r="AS1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="41"/>
+      <c r="P1" s="41"/>
+      <c r="Q1" s="41"/>
+      <c r="R1" s="41"/>
+      <c r="S1" s="41"/>
+      <c r="T1" s="55"/>
+      <c r="U1" s="56"/>
+      <c r="V1" s="40"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10"/>
+      <c r="Z1" s="10"/>
+      <c r="AA1" s="10"/>
+      <c r="AB1" s="10"/>
+      <c r="AC1" s="63"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="10"/>
+      <c r="AF1" s="10"/>
+      <c r="AG1" s="40"/>
+      <c r="AH1" s="10"/>
+      <c r="AI1" s="10"/>
+      <c r="AJ1" s="10"/>
+      <c r="AK1" s="10"/>
+      <c r="AL1" s="10"/>
+      <c r="AM1" s="10"/>
+      <c r="AN1" s="10"/>
+      <c r="AO1" s="10"/>
+      <c r="AP1" s="10"/>
+      <c r="AQ1" s="10"/>
+      <c r="AR1" s="40"/>
+      <c r="AS1" s="10"/>
     </row>
     <row r="2" spans="1:45">
-      <c r="A2" s="10"/>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="47"/>
-      <c r="P2" s="47"/>
-      <c r="Q2" s="47"/>
-      <c r="R2" s="58"/>
-      <c r="S2" s="47"/>
-      <c r="T2" s="59"/>
-      <c r="U2" s="59"/>
-      <c r="V2" s="45"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="65"/>
-      <c r="Z2" s="12"/>
-      <c r="AA2" s="66"/>
-      <c r="AB2" s="67"/>
-      <c r="AC2" s="67"/>
-      <c r="AD2" s="68" t="s">
+      <c r="A2" s="12"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="44"/>
+      <c r="N2" s="44"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="46"/>
+      <c r="Q2" s="46"/>
+      <c r="R2" s="57"/>
+      <c r="S2" s="46"/>
+      <c r="T2" s="58"/>
+      <c r="U2" s="58"/>
+      <c r="V2" s="44"/>
+      <c r="W2" s="14"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="64"/>
+      <c r="Z2" s="14"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="66"/>
+      <c r="AC2" s="66"/>
+      <c r="AD2" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="AE2" s="69"/>
-      <c r="AF2" s="70"/>
-      <c r="AG2" s="45"/>
-      <c r="AH2" s="12"/>
-      <c r="AI2" s="12"/>
-      <c r="AJ2" s="12"/>
-      <c r="AK2" s="14"/>
-      <c r="AL2" s="12"/>
-      <c r="AM2" s="12"/>
-      <c r="AN2" s="12"/>
-      <c r="AP2" s="12"/>
-      <c r="AQ2" s="12"/>
-      <c r="AR2" s="77"/>
-      <c r="AS2" s="11"/>
+      <c r="AE2" s="68"/>
+      <c r="AF2" s="69"/>
+      <c r="AG2" s="44"/>
+      <c r="AH2" s="14"/>
+      <c r="AI2" s="14"/>
+      <c r="AJ2" s="14"/>
+      <c r="AK2" s="16"/>
+      <c r="AL2" s="14"/>
+      <c r="AM2" s="14"/>
+      <c r="AN2" s="14"/>
+      <c r="AP2" s="14"/>
+      <c r="AQ2" s="14"/>
+      <c r="AR2" s="76"/>
+      <c r="AS2" s="13"/>
     </row>
     <row r="3" ht="20" spans="1:45">
-      <c r="A3" s="16"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="18">
+      <c r="A3" s="18"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="20">
         <v>13</v>
       </c>
-      <c r="E3" s="18">
-        <v>14</v>
-      </c>
-      <c r="F3" s="18">
-        <v>15</v>
-      </c>
-      <c r="G3" s="18">
+      <c r="E3" s="20">
+        <v>14</v>
+      </c>
+      <c r="F3" s="20">
+        <v>15</v>
+      </c>
+      <c r="G3" s="20">
         <v>16</v>
       </c>
-      <c r="H3" s="18">
+      <c r="H3" s="20">
         <v>17</v>
       </c>
-      <c r="I3" s="18">
+      <c r="I3" s="20">
         <v>18</v>
       </c>
-      <c r="J3" s="18">
+      <c r="J3" s="20">
         <v>19</v>
       </c>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18">
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20">
         <v>20</v>
       </c>
-      <c r="P3" s="18">
+      <c r="P3" s="20">
         <v>21</v>
       </c>
-      <c r="Q3" s="18">
+      <c r="Q3" s="20">
         <v>22</v>
       </c>
-      <c r="R3" s="18">
+      <c r="R3" s="20">
         <v>23</v>
       </c>
-      <c r="S3" s="18">
+      <c r="S3" s="20">
         <v>24</v>
       </c>
-      <c r="T3" s="18">
+      <c r="T3" s="20">
         <v>25</v>
       </c>
-      <c r="U3" s="18">
+      <c r="U3" s="20">
         <v>26</v>
       </c>
-      <c r="V3" s="18"/>
-      <c r="W3" s="18"/>
-      <c r="X3" s="18"/>
-      <c r="Y3" s="18"/>
-      <c r="Z3" s="18">
+      <c r="V3" s="20"/>
+      <c r="W3" s="20"/>
+      <c r="X3" s="20"/>
+      <c r="Y3" s="20"/>
+      <c r="Z3" s="20">
         <v>27</v>
       </c>
-      <c r="AA3" s="18">
+      <c r="AA3" s="20">
         <v>28</v>
       </c>
-      <c r="AB3" s="18">
+      <c r="AB3" s="20">
         <v>29</v>
       </c>
-      <c r="AC3" s="18">
+      <c r="AC3" s="20">
         <v>30</v>
       </c>
-      <c r="AD3" s="18">
+      <c r="AD3" s="20">
         <v>1</v>
       </c>
-      <c r="AE3" s="18">
+      <c r="AE3" s="20">
         <v>2</v>
       </c>
-      <c r="AF3" s="18">
+      <c r="AF3" s="20">
         <v>3</v>
       </c>
-      <c r="AG3" s="18"/>
-      <c r="AH3" s="18"/>
-      <c r="AI3" s="18"/>
-      <c r="AJ3" s="18"/>
-      <c r="AK3" s="18">
+      <c r="AG3" s="20"/>
+      <c r="AH3" s="20"/>
+      <c r="AI3" s="20"/>
+      <c r="AJ3" s="20"/>
+      <c r="AK3" s="20">
         <v>4</v>
       </c>
-      <c r="AL3" s="18">
+      <c r="AL3" s="20">
         <v>5</v>
       </c>
-      <c r="AM3" s="18">
+      <c r="AM3" s="20">
         <v>6</v>
       </c>
-      <c r="AN3" s="18">
+      <c r="AN3" s="20">
         <v>7</v>
       </c>
-      <c r="AO3" s="18">
+      <c r="AO3" s="20">
         <v>8</v>
       </c>
-      <c r="AP3" s="18">
+      <c r="AP3" s="20">
         <v>9</v>
       </c>
-      <c r="AQ3" s="18">
+      <c r="AQ3" s="20">
         <v>10</v>
       </c>
-      <c r="AR3" s="11"/>
-      <c r="AS3" s="17"/>
+      <c r="AR3" s="13"/>
+      <c r="AS3" s="19"/>
     </row>
     <row r="4" ht="14.5" spans="1:45">
-      <c r="A4" s="19"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="22" t="s">
+      <c r="A4" s="21"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="23" t="s">
+      <c r="G4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="23" t="s">
+      <c r="H4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="23" t="s">
+      <c r="I4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="22" t="s">
+      <c r="J4" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="K4" s="21"/>
-      <c r="L4" s="21"/>
-      <c r="M4" s="21"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22" t="s">
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="P4" s="23" t="s">
+      <c r="P4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="Q4" s="23" t="s">
+      <c r="Q4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="R4" s="23" t="s">
+      <c r="R4" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="S4" s="23" t="s">
+      <c r="S4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="T4" s="23" t="s">
+      <c r="T4" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="U4" s="22" t="s">
+      <c r="U4" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="V4" s="60"/>
-      <c r="W4" s="60"/>
-      <c r="X4" s="21"/>
-      <c r="Y4" s="22"/>
-      <c r="Z4" s="71" t="s">
+      <c r="V4" s="59"/>
+      <c r="W4" s="59"/>
+      <c r="X4" s="23"/>
+      <c r="Y4" s="24"/>
+      <c r="Z4" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="AA4" s="72" t="s">
+      <c r="AA4" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="AB4" s="72" t="s">
+      <c r="AB4" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="AC4" s="72" t="s">
+      <c r="AC4" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="AD4" s="72" t="s">
+      <c r="AD4" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="AE4" s="72" t="s">
+      <c r="AE4" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="AF4" s="71" t="s">
+      <c r="AF4" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="AG4" s="21"/>
-      <c r="AH4" s="20"/>
-      <c r="AI4" s="21"/>
-      <c r="AJ4" s="21"/>
-      <c r="AK4" s="71" t="s">
+      <c r="AG4" s="23"/>
+      <c r="AH4" s="22"/>
+      <c r="AI4" s="23"/>
+      <c r="AJ4" s="23"/>
+      <c r="AK4" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="AL4" s="72" t="s">
+      <c r="AL4" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="AM4" s="72" t="s">
+      <c r="AM4" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="AN4" s="72" t="s">
+      <c r="AN4" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="AO4" s="72" t="s">
+      <c r="AO4" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="AP4" s="72" t="s">
+      <c r="AP4" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="AQ4" s="71" t="s">
+      <c r="AQ4" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="AR4" s="21"/>
-      <c r="AS4" s="20"/>
+      <c r="AR4" s="23"/>
+      <c r="AS4" s="22"/>
     </row>
     <row r="5" ht="14.5" spans="1:45">
-      <c r="A5" s="10"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="49"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="50"/>
-      <c r="O5" s="50"/>
-      <c r="P5" s="50"/>
-      <c r="Q5" s="50"/>
-      <c r="R5" s="50"/>
-      <c r="S5" s="50"/>
-      <c r="T5" s="50"/>
-      <c r="U5" s="51"/>
-      <c r="V5" s="51"/>
-      <c r="W5" s="61"/>
-      <c r="X5" s="21"/>
-      <c r="Y5" s="26"/>
-      <c r="Z5" s="26"/>
-      <c r="AA5" s="26"/>
-      <c r="AB5" s="26"/>
-      <c r="AC5" s="26"/>
-      <c r="AD5" s="26"/>
-      <c r="AE5" s="26"/>
-      <c r="AF5" s="48"/>
-      <c r="AG5" s="48"/>
-      <c r="AH5" s="73"/>
-      <c r="AI5" s="21"/>
-      <c r="AJ5" s="74"/>
-      <c r="AK5" s="74"/>
-      <c r="AL5" s="74"/>
-      <c r="AM5" s="74"/>
-      <c r="AN5" s="74"/>
-      <c r="AO5" s="74"/>
-      <c r="AP5" s="74"/>
-      <c r="AQ5" s="74"/>
-      <c r="AR5" s="48"/>
-      <c r="AS5" s="24"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="47"/>
+      <c r="L5" s="48"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="49"/>
+      <c r="O5" s="49"/>
+      <c r="P5" s="49"/>
+      <c r="Q5" s="49"/>
+      <c r="R5" s="49"/>
+      <c r="S5" s="49"/>
+      <c r="T5" s="49"/>
+      <c r="U5" s="50"/>
+      <c r="V5" s="50"/>
+      <c r="W5" s="60"/>
+      <c r="X5" s="23"/>
+      <c r="Y5" s="28"/>
+      <c r="Z5" s="28"/>
+      <c r="AA5" s="28"/>
+      <c r="AB5" s="28"/>
+      <c r="AC5" s="28"/>
+      <c r="AD5" s="28"/>
+      <c r="AE5" s="28"/>
+      <c r="AF5" s="47"/>
+      <c r="AG5" s="47"/>
+      <c r="AH5" s="72"/>
+      <c r="AI5" s="23"/>
+      <c r="AJ5" s="73"/>
+      <c r="AK5" s="73"/>
+      <c r="AL5" s="73"/>
+      <c r="AM5" s="73"/>
+      <c r="AN5" s="73"/>
+      <c r="AO5" s="73"/>
+      <c r="AP5" s="73"/>
+      <c r="AQ5" s="73"/>
+      <c r="AR5" s="47"/>
+      <c r="AS5" s="26"/>
     </row>
     <row r="6" ht="18.5" spans="1:45">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="29">
         <v>6</v>
       </c>
-      <c r="D6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="30" t="s">
+      <c r="D6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="29" t="s">
+      <c r="F6" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="I6" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="K6" s="51">
-        <v>40</v>
-      </c>
-      <c r="L6" s="52"/>
-      <c r="M6" s="27" t="s">
+      <c r="G6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="50">
+        <v>40</v>
+      </c>
+      <c r="L6" s="51"/>
+      <c r="M6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="N6" s="32">
+      <c r="N6" s="33">
         <v>5</v>
       </c>
-      <c r="O6" s="29" t="s">
+      <c r="O6" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="P6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q6" s="30" t="s">
+      <c r="P6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q6" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="R6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="S6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="T6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="U6" s="53" t="s">
+      <c r="R6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="S6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="T6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="U6" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="V6" s="51">
-        <v>40</v>
-      </c>
-      <c r="W6" s="62"/>
-      <c r="X6" s="27" t="s">
+      <c r="V6" s="50">
+        <v>40</v>
+      </c>
+      <c r="W6" s="61"/>
+      <c r="X6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="Y6" s="32"/>
-      <c r="Z6" s="33" t="s">
+      <c r="Y6" s="33"/>
+      <c r="Z6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AA6" s="33" t="s">
+      <c r="AA6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AB6" s="28" t="s">
+      <c r="AB6" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="AC6" s="30" t="s">
+      <c r="AC6" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AD6" s="29" t="s">
+      <c r="AD6" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AE6" s="33" t="s">
+      <c r="AE6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AF6" s="33" t="s">
+      <c r="AF6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AG6" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH6" s="48"/>
-      <c r="AI6" s="27" t="s">
+      <c r="AG6" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH6" s="47"/>
+      <c r="AI6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="AJ6" s="32"/>
-      <c r="AK6" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="AL6" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AM6" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AN6" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AO6" s="30" t="s">
+      <c r="AJ6" s="33"/>
+      <c r="AK6" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="AL6" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AM6" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AN6" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AO6" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AP6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AQ6" s="53" t="s">
+      <c r="AP6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AQ6" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="AR6" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS6" s="78"/>
+      <c r="AR6" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS6" s="77"/>
     </row>
     <row r="7" ht="18.5" spans="1:45">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="32">
+      <c r="C7" s="33">
         <v>5</v>
       </c>
-      <c r="D7" s="29" t="s">
+      <c r="D7" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="30" t="s">
+      <c r="E7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="H7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="J7" s="53" t="s">
+      <c r="G7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="51">
-        <v>40</v>
-      </c>
-      <c r="L7" s="52"/>
-      <c r="M7" s="27" t="s">
+      <c r="K7" s="50">
+        <v>40</v>
+      </c>
+      <c r="L7" s="51"/>
+      <c r="M7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="32"/>
-      <c r="O7" s="33" t="s">
+      <c r="N7" s="33"/>
+      <c r="O7" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="P7" s="33" t="s">
+      <c r="P7" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="Q7" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="R7" s="30" t="s">
+      <c r="Q7" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="R7" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="S7" s="29" t="s">
+      <c r="S7" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="T7" s="33" t="s">
+      <c r="T7" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="U7" s="33" t="s">
+      <c r="U7" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="V7" s="51">
-        <v>40</v>
-      </c>
-      <c r="W7" s="62"/>
-      <c r="X7" s="27" t="s">
+      <c r="V7" s="50">
+        <v>40</v>
+      </c>
+      <c r="W7" s="61"/>
+      <c r="X7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="Y7" s="32"/>
-      <c r="Z7" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA7" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AB7" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC7" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE7" s="30" t="s">
+      <c r="Y7" s="33"/>
+      <c r="Z7" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="AA7" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AB7" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC7" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE7" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AF7" s="53" t="s">
+      <c r="AF7" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="AG7" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH7" s="75"/>
-      <c r="AI7" s="27" t="s">
+      <c r="AG7" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH7" s="74"/>
+      <c r="AI7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="AJ7" s="28"/>
-      <c r="AK7" s="34" t="s">
+      <c r="AJ7" s="29"/>
+      <c r="AK7" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="AL7" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AM7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AN7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AO7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP7" s="29" t="s">
+      <c r="AL7" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AM7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO7" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP7" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="AQ7" s="54" t="s">
+      <c r="AQ7" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="AR7" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS7" s="78"/>
+      <c r="AR7" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS7" s="77"/>
     </row>
     <row r="8" ht="18.5" spans="1:45">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="33" t="s">
+      <c r="C8" s="33"/>
+      <c r="D8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="33" t="s">
+      <c r="E8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="30" t="s">
+      <c r="F8" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="H8" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="33" t="s">
+      <c r="I8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="33" t="s">
+      <c r="J8" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="51">
-        <v>40</v>
-      </c>
-      <c r="L8" s="52"/>
-      <c r="M8" s="27" t="s">
+      <c r="K8" s="50">
+        <v>40</v>
+      </c>
+      <c r="L8" s="51"/>
+      <c r="M8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="N8" s="32"/>
-      <c r="O8" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="P8" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q8" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="R8" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="S8" s="30" t="s">
+      <c r="N8" s="33"/>
+      <c r="O8" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="P8" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q8" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="R8" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="S8" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="T8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="U8" s="53" t="s">
+      <c r="T8" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="U8" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="V8" s="51">
-        <v>40</v>
-      </c>
-      <c r="W8" s="62"/>
-      <c r="X8" s="27" t="s">
+      <c r="V8" s="50">
+        <v>40</v>
+      </c>
+      <c r="W8" s="61"/>
+      <c r="X8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Y8" s="28"/>
-      <c r="Z8" s="34" t="s">
+      <c r="Y8" s="29"/>
+      <c r="Z8" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="AA8" s="28" t="s">
+      <c r="AA8" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="AB8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE8" s="29" t="s">
+      <c r="AB8" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC8" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD8" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE8" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="AF8" s="54" t="s">
+      <c r="AF8" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="AG8" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH8" s="75"/>
-      <c r="AI8" s="27" t="s">
+      <c r="AG8" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH8" s="74"/>
+      <c r="AI8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="AJ8" s="28"/>
-      <c r="AK8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL8" s="30" t="s">
+      <c r="AJ8" s="29"/>
+      <c r="AK8" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL8" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AM8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AN8" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AO8" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AP8" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AQ8" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AR8" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS8" s="78"/>
+      <c r="AM8" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN8" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO8" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AP8" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AQ8" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AR8" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS8" s="77"/>
     </row>
     <row r="9" ht="18.5" spans="1:45">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="29" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="30" t="s">
+      <c r="C9" s="33"/>
+      <c r="D9" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="J9" s="53" t="s">
+      <c r="I9" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="K9" s="51">
-        <v>40</v>
-      </c>
-      <c r="L9" s="52"/>
-      <c r="M9" s="27" t="s">
+      <c r="K9" s="50">
+        <v>40</v>
+      </c>
+      <c r="L9" s="51"/>
+      <c r="M9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="N9" s="28"/>
-      <c r="O9" s="34" t="s">
+      <c r="N9" s="29"/>
+      <c r="O9" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="P9" s="28" t="s">
+      <c r="P9" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="Q9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="R9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="S9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="T9" s="28" t="s">
+      <c r="Q9" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="T9" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="U9" s="54" t="s">
+      <c r="U9" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="V9" s="51">
-        <v>40</v>
-      </c>
-      <c r="W9" s="62"/>
-      <c r="X9" s="27" t="s">
+      <c r="V9" s="50">
+        <v>40</v>
+      </c>
+      <c r="W9" s="61"/>
+      <c r="X9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Y9" s="28"/>
-      <c r="Z9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AA9" s="30" t="s">
+      <c r="Y9" s="29"/>
+      <c r="Z9" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA9" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AB9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC9" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AD9" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE9" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AF9" s="28" t="s">
+      <c r="AB9" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC9" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AD9" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AE9" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AF9" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="AG9" s="51">
+      <c r="AG9" s="50">
         <v>32</v>
       </c>
-      <c r="AH9" s="75"/>
-      <c r="AI9" s="27" t="s">
+      <c r="AH9" s="74"/>
+      <c r="AI9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="AJ9" s="35"/>
-      <c r="AK9" s="33" t="s">
+      <c r="AJ9" s="36"/>
+      <c r="AK9" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AL9" s="33" t="s">
+      <c r="AL9" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AM9" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AN9" s="28" t="s">
+      <c r="AM9" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AN9" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="AO9" s="36" t="s">
+      <c r="AO9" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AP9" s="36" t="s">
+      <c r="AP9" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AQ9" s="36" t="s">
+      <c r="AQ9" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="AR9" s="51">
+      <c r="AR9" s="50">
         <v>48</v>
       </c>
-      <c r="AS9" s="78"/>
+      <c r="AS9" s="77"/>
     </row>
     <row r="10" ht="18.5" spans="1:45">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="34" t="s">
+      <c r="C10" s="29"/>
+      <c r="D10" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="28" t="s">
+      <c r="E10" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I10" s="30" t="s">
+      <c r="F10" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="J10" s="54" t="s">
+      <c r="J10" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="K10" s="51">
-        <v>40</v>
-      </c>
-      <c r="L10" s="52"/>
-      <c r="M10" s="27" t="s">
+      <c r="K10" s="50">
+        <v>40</v>
+      </c>
+      <c r="L10" s="51"/>
+      <c r="M10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N10" s="28"/>
-      <c r="O10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="P10" s="28" t="s">
+      <c r="N10" s="29"/>
+      <c r="O10" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="P10" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="Q10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="R10" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="S10" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="T10" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="U10" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="V10" s="51">
+      <c r="Q10" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="R10" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="S10" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="T10" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="U10" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="V10" s="50">
         <v>32</v>
       </c>
-      <c r="W10" s="62"/>
-      <c r="X10" s="27" t="s">
+      <c r="W10" s="61"/>
+      <c r="X10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="Y10" s="35"/>
-      <c r="Z10" s="33" t="s">
+      <c r="Y10" s="36"/>
+      <c r="Z10" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AA10" s="33" t="s">
+      <c r="AA10" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AB10" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AC10" s="30" t="s">
+      <c r="AB10" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AC10" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AD10" s="33" t="s">
+      <c r="AD10" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AE10" s="33" t="s">
+      <c r="AE10" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AF10" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AG10" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH10" s="75"/>
-      <c r="AI10" s="27" t="s">
+      <c r="AF10" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AG10" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH10" s="74"/>
+      <c r="AI10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="AJ10" s="28">
+      <c r="AJ10" s="29">
         <v>1</v>
       </c>
-      <c r="AK10" s="37" t="s">
+      <c r="AK10" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="AL10" s="37" t="s">
+      <c r="AL10" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="AM10" s="37" t="s">
+      <c r="AM10" s="38" t="s">
         <v>16</v>
       </c>
       <c r="AN10" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="AO10" s="37" t="s">
+      <c r="AO10" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="AP10" s="37" t="s">
+      <c r="AP10" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="AQ10" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="AR10" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS10" s="78"/>
+      <c r="AQ10" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="AR10" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS10" s="77"/>
     </row>
     <row r="11" ht="18.5" spans="1:45">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="30" t="s">
+      <c r="C11" s="29"/>
+      <c r="D11" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="28" t="s">
+      <c r="F11" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="K11" s="51">
-        <v>40</v>
-      </c>
-      <c r="L11" s="52"/>
-      <c r="M11" s="27" t="s">
+      <c r="I11" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="K11" s="50">
+        <v>40</v>
+      </c>
+      <c r="L11" s="51"/>
+      <c r="M11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="N11" s="35"/>
-      <c r="O11" s="36" t="s">
+      <c r="N11" s="36"/>
+      <c r="O11" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="P11" s="36" t="s">
+      <c r="P11" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="Q11" s="36" t="s">
+      <c r="Q11" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="R11" s="36" t="s">
+      <c r="R11" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="S11" s="36" t="s">
+      <c r="S11" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="T11" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="U11" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="V11" s="51">
-        <v>40</v>
-      </c>
-      <c r="W11" s="63"/>
-      <c r="X11" s="27" t="s">
+      <c r="T11" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="U11" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="V11" s="50">
+        <v>40</v>
+      </c>
+      <c r="W11" s="62"/>
+      <c r="X11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="Y11" s="28">
+      <c r="Y11" s="29">
         <v>1</v>
       </c>
-      <c r="Z11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AA11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC11" s="29" t="s">
+      <c r="Z11" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA11" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB11" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC11" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="AD11" s="54" t="s">
+      <c r="AD11" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="AE11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AF11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AG11" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH11" s="75"/>
-      <c r="AI11" s="27" t="s">
+      <c r="AE11" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF11" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG11" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH11" s="74"/>
+      <c r="AI11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AJ11" s="28"/>
-      <c r="AK11" s="30" t="s">
+      <c r="AJ11" s="29"/>
+      <c r="AK11" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AL11" s="34" t="s">
+      <c r="AL11" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="AM11" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AN11" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AO11" s="29" t="s">
+      <c r="AM11" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AN11" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AO11" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AP11" s="55" t="s">
+      <c r="AP11" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="AQ11" s="53" t="s">
+      <c r="AQ11" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="AR11" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS11" s="78"/>
+      <c r="AR11" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS11" s="77"/>
     </row>
     <row r="12" ht="18.5" spans="1:45">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="27" t="s">
+      <c r="B12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36" t="s">
+      <c r="C12" s="36"/>
+      <c r="D12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="36" t="s">
+      <c r="E12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="36" t="s">
+      <c r="F12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="36" t="s">
+      <c r="G12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="H12" s="36" t="s">
+      <c r="H12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="I12" s="36" t="s">
+      <c r="I12" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="J12" s="36" t="s">
+      <c r="J12" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="K12" s="51">
+      <c r="K12" s="50">
         <v>48</v>
       </c>
-      <c r="L12" s="52"/>
-      <c r="M12" s="27" t="s">
+      <c r="L12" s="51"/>
+      <c r="M12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="N12" s="28">
+      <c r="N12" s="29">
         <v>1</v>
       </c>
-      <c r="O12" s="37" t="s">
+      <c r="O12" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="P12" s="37" t="s">
+      <c r="P12" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="Q12" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="R12" s="28" t="s">
+      <c r="Q12" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="R12" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="S12" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="T12" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="U12" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="V12" s="51">
+      <c r="S12" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="T12" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="U12" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="V12" s="50">
         <v>32</v>
       </c>
-      <c r="W12" s="62"/>
-      <c r="X12" s="27" t="s">
+      <c r="W12" s="61"/>
+      <c r="X12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="Y12" s="28"/>
-      <c r="Z12" s="30" t="s">
+      <c r="Y12" s="29"/>
+      <c r="Z12" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AA12" s="34" t="s">
+      <c r="AA12" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="AB12" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AC12" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AD12" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE12" s="55" t="s">
+      <c r="AB12" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC12" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD12" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE12" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="AF12" s="36" t="s">
+      <c r="AF12" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="AG12" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH12" s="75"/>
-      <c r="AI12" s="27" t="s">
+      <c r="AG12" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH12" s="74"/>
+      <c r="AI12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AJ12" s="28">
+      <c r="AJ12" s="29">
         <v>4</v>
       </c>
-      <c r="AK12" s="36" t="s">
+      <c r="AK12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AL12" s="36" t="s">
+      <c r="AL12" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AM12" s="36" t="s">
+      <c r="AM12" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="AN12" s="36" t="s">
+      <c r="AN12" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="AO12" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP12" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AQ12" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AR12" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS12" s="78"/>
+      <c r="AO12" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP12" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AQ12" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AR12" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS12" s="77"/>
     </row>
     <row r="13" ht="18.5" spans="1:45">
-      <c r="A13" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="27" t="s">
+      <c r="A13" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="29">
         <v>1</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="37" t="s">
+      <c r="E13" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" s="37" t="s">
+      <c r="F13" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="37" t="s">
+      <c r="H13" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="37" t="s">
+      <c r="I13" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="K13" s="51">
-        <v>40</v>
-      </c>
-      <c r="L13" s="52"/>
-      <c r="M13" s="27" t="s">
+      <c r="J13" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="K13" s="50">
+        <v>40</v>
+      </c>
+      <c r="L13" s="51"/>
+      <c r="M13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="N13" s="28"/>
-      <c r="O13" s="30" t="s">
+      <c r="N13" s="29"/>
+      <c r="O13" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="P13" s="34" t="s">
+      <c r="P13" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="Q13" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="R13" s="28" t="s">
+      <c r="Q13" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="R13" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="S13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="T13" s="55" t="s">
+      <c r="S13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="T13" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="U13" s="29" t="s">
+      <c r="U13" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="V13" s="51">
-        <v>40</v>
-      </c>
-      <c r="W13" s="62"/>
-      <c r="X13" s="27" t="s">
+      <c r="V13" s="50">
+        <v>40</v>
+      </c>
+      <c r="W13" s="61"/>
+      <c r="X13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="Y13" s="28">
+      <c r="Y13" s="29">
         <v>4</v>
       </c>
-      <c r="Z13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AA13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB13" s="30" t="s">
+      <c r="Z13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB13" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AC13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AF13" s="28" t="s">
+      <c r="AC13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF13" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="AG13" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH13" s="75"/>
-      <c r="AI13" s="27" t="s">
+      <c r="AG13" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH13" s="74"/>
+      <c r="AI13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AJ13" s="32"/>
-      <c r="AK13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AM13" s="33" t="s">
+      <c r="AJ13" s="33"/>
+      <c r="AK13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL13" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM13" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AN13" s="33" t="s">
+      <c r="AN13" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AO13" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AP13" s="29" t="s">
+      <c r="AO13" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AP13" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="AQ13" s="54" t="s">
+      <c r="AQ13" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="AR13" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS13" s="78"/>
+      <c r="AR13" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS13" s="77"/>
     </row>
     <row r="14" ht="17.5" spans="1:45">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="30" t="s">
+      <c r="C14" s="29"/>
+      <c r="D14" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="34" t="s">
+      <c r="E14" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="G14" s="28" t="s">
+      <c r="F14" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I14" s="55" t="s">
+      <c r="H14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" s="54" t="s">
         <v>37</v>
       </c>
-      <c r="J14" s="29" t="s">
+      <c r="J14" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="K14" s="51">
-        <v>40</v>
-      </c>
-      <c r="L14" s="52"/>
-      <c r="M14" s="38" t="s">
+      <c r="K14" s="50">
+        <v>40</v>
+      </c>
+      <c r="L14" s="51"/>
+      <c r="M14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="N14" s="28">
+      <c r="N14" s="29">
         <v>4</v>
       </c>
-      <c r="O14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="P14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q14" s="30" t="s">
+      <c r="O14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="P14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q14" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="R14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="S14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="T14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="U14" s="29" t="s">
+      <c r="R14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="S14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="T14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="U14" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="V14" s="51">
-        <v>40</v>
-      </c>
-      <c r="W14" s="62"/>
-      <c r="X14" s="38" t="s">
+      <c r="V14" s="50">
+        <v>40</v>
+      </c>
+      <c r="W14" s="61"/>
+      <c r="X14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="Y14" s="32"/>
-      <c r="Z14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AA14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB14" s="33" t="s">
+      <c r="Y14" s="33"/>
+      <c r="Z14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB14" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AC14" s="33" t="s">
+      <c r="AC14" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="AD14" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE14" s="30" t="s">
+      <c r="AD14" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AE14" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AF14" s="54" t="s">
+      <c r="AF14" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="AG14" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH14" s="75"/>
-      <c r="AI14" s="38" t="s">
+      <c r="AG14" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH14" s="74"/>
+      <c r="AI14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="AJ14" s="28">
+      <c r="AJ14" s="29">
         <v>2</v>
       </c>
-      <c r="AK14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL14" s="29" t="s">
+      <c r="AK14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL14" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="AM14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AN14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AO14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP14" s="29" t="s">
+      <c r="AM14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP14" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AQ14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AR14" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS14" s="78"/>
+      <c r="AQ14" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AR14" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS14" s="77"/>
     </row>
     <row r="15" ht="18.5" spans="1:45">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="27" t="s">
+      <c r="B15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="28">
+      <c r="C15" s="29">
         <v>4</v>
       </c>
-      <c r="D15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="30" t="s">
+      <c r="D15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="H15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="J15" s="29" t="s">
+      <c r="G15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="J15" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="K15" s="51">
+      <c r="K15" s="50">
         <v>32</v>
       </c>
-      <c r="L15" s="52"/>
-      <c r="M15" s="27" t="s">
+      <c r="L15" s="51"/>
+      <c r="M15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="N15" s="32"/>
-      <c r="O15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="P15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q15" s="33" t="s">
+      <c r="N15" s="33"/>
+      <c r="O15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="P15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q15" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="R15" s="33" t="s">
+      <c r="R15" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="S15" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="T15" s="30" t="s">
+      <c r="S15" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="T15" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="U15" s="54" t="s">
+      <c r="U15" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="V15" s="51">
-        <v>40</v>
-      </c>
-      <c r="W15" s="62"/>
-      <c r="X15" s="27" t="s">
+      <c r="V15" s="50">
+        <v>40</v>
+      </c>
+      <c r="W15" s="61"/>
+      <c r="X15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="Y15" s="28">
+      <c r="Y15" s="29">
         <v>2</v>
       </c>
-      <c r="Z15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AA15" s="29" t="s">
+      <c r="Z15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA15" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="AB15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC15" s="29" t="s">
+      <c r="AB15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC15" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AD15" s="54" t="s">
+      <c r="AD15" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="AE15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AF15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AG15" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH15" s="75"/>
-      <c r="AI15" s="27" t="s">
+      <c r="AE15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG15" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH15" s="74"/>
+      <c r="AI15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="AJ15" s="32"/>
-      <c r="AK15" s="29" t="s">
+      <c r="AJ15" s="33"/>
+      <c r="AK15" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AL15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AM15" s="30" t="s">
+      <c r="AL15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM15" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AN15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AO15" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AP15" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AQ15" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AR15" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS15" s="78"/>
+      <c r="AN15" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO15" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AP15" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AQ15" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AR15" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS15" s="77"/>
     </row>
     <row r="16" ht="18.5" spans="1:45">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="32"/>
-      <c r="D16" s="36" t="s">
+      <c r="C16" s="33"/>
+      <c r="D16" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="E16" s="36" t="s">
+      <c r="E16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="36" t="s">
+      <c r="F16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="36" t="s">
+      <c r="G16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="H16" s="36" t="s">
+      <c r="H16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="I16" s="36" t="s">
+      <c r="I16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="J16" s="36" t="s">
+      <c r="J16" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="K16" s="51">
-        <v>40</v>
-      </c>
-      <c r="L16" s="52"/>
-      <c r="M16" s="27" t="s">
+      <c r="K16" s="50">
+        <v>40</v>
+      </c>
+      <c r="L16" s="51"/>
+      <c r="M16" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="N16" s="28">
+      <c r="N16" s="29">
         <v>2</v>
       </c>
-      <c r="O16" s="36" t="s">
+      <c r="O16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="P16" s="36" t="s">
+      <c r="P16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="Q16" s="36" t="s">
+      <c r="Q16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="R16" s="36" t="s">
+      <c r="R16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="S16" s="36" t="s">
+      <c r="S16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="T16" s="36" t="s">
+      <c r="T16" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="U16" s="36" t="s">
+      <c r="U16" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="V16" s="51">
-        <v>40</v>
-      </c>
-      <c r="W16" s="62"/>
-      <c r="X16" s="27" t="s">
+      <c r="V16" s="50">
+        <v>40</v>
+      </c>
+      <c r="W16" s="61"/>
+      <c r="X16" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="Y16" s="32"/>
-      <c r="Z16" s="36" t="s">
+      <c r="Y16" s="33"/>
+      <c r="Z16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AA16" s="36" t="s">
+      <c r="AA16" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AB16" s="36" t="s">
+      <c r="AB16" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="AC16" s="36" t="s">
+      <c r="AC16" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="AD16" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AE16" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AF16" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AG16" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH16" s="75"/>
-      <c r="AI16" s="27" t="s">
+      <c r="AD16" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE16" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF16" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AG16" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH16" s="74"/>
+      <c r="AI16" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="AJ16" s="32"/>
-      <c r="AK16" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AL16" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AM16" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AN16" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AO16" s="28" t="s">
+      <c r="AJ16" s="33"/>
+      <c r="AK16" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AL16" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AM16" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN16" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AO16" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="AP16" s="53" t="s">
+      <c r="AP16" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="AQ16" s="29" t="s">
+      <c r="AQ16" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="AR16" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS16" s="78"/>
+      <c r="AR16" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS16" s="77"/>
     </row>
     <row r="17" ht="18.5" spans="1:45">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="29">
         <v>2</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="D17" s="30" t="s">
         <v>11</v>
       </c>
       <c r="E17" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="37" t="s">
+      <c r="F17" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="G17" s="37" t="s">
+      <c r="G17" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="37" t="s">
+      <c r="H17" s="38" t="s">
         <v>15</v>
       </c>
       <c r="I17" s="39" t="s">
@@ -3393,591 +3392,591 @@
       <c r="J17" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="K17" s="51">
-        <v>40</v>
-      </c>
-      <c r="L17" s="52"/>
-      <c r="M17" s="27" t="s">
+      <c r="K17" s="50">
+        <v>40</v>
+      </c>
+      <c r="L17" s="51"/>
+      <c r="M17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="N17" s="32"/>
-      <c r="O17" s="29" t="s">
+      <c r="N17" s="33"/>
+      <c r="O17" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="P17" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q17" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="R17" s="30" t="s">
+      <c r="P17" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q17" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="R17" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="S17" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="T17" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="U17" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="V17" s="51">
-        <v>40</v>
-      </c>
-      <c r="W17" s="62"/>
-      <c r="X17" s="27" t="s">
+      <c r="S17" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="T17" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="U17" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="V17" s="50">
+        <v>40</v>
+      </c>
+      <c r="W17" s="61"/>
+      <c r="X17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="Y17" s="32"/>
-      <c r="Z17" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AA17" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AB17" s="30" t="s">
+      <c r="Y17" s="33"/>
+      <c r="Z17" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AA17" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AB17" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AC17" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AD17" s="28" t="s">
+      <c r="AC17" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AD17" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="AE17" s="53" t="s">
+      <c r="AE17" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="AF17" s="53" t="s">
+      <c r="AF17" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="AG17" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH17" s="75"/>
-      <c r="AI17" s="27" t="s">
+      <c r="AG17" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH17" s="74"/>
+      <c r="AI17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="AJ17" s="32">
+      <c r="AJ17" s="33">
         <v>3</v>
       </c>
-      <c r="AK17" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL17" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AM17" s="29" t="s">
+      <c r="AK17" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL17" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM17" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="AN17" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AO17" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP17" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AQ17" s="29" t="s">
+      <c r="AN17" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO17" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP17" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AQ17" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AR17" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS17" s="79"/>
+      <c r="AR17" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS17" s="78"/>
     </row>
     <row r="18" ht="18.5" spans="1:45">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="28" t="s">
+      <c r="C18" s="33"/>
+      <c r="D18" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="E18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="30" t="s">
+      <c r="E18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="H18" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="I18" s="28" t="s">
+      <c r="H18" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="I18" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="J18" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="K18" s="51">
-        <v>40</v>
-      </c>
-      <c r="L18" s="52"/>
-      <c r="M18" s="27" t="s">
+      <c r="J18" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="K18" s="50">
+        <v>40</v>
+      </c>
+      <c r="L18" s="51"/>
+      <c r="M18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="N18" s="32"/>
-      <c r="O18" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="P18" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q18" s="29" t="s">
+      <c r="N18" s="33"/>
+      <c r="O18" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="P18" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q18" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="R18" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="S18" s="28" t="s">
+      <c r="R18" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="S18" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="T18" s="53" t="s">
+      <c r="T18" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="U18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="V18" s="51">
-        <v>40</v>
-      </c>
-      <c r="W18" s="62"/>
-      <c r="X18" s="27" t="s">
+      <c r="U18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="V18" s="50">
+        <v>40</v>
+      </c>
+      <c r="W18" s="61"/>
+      <c r="X18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="Y18" s="32">
+      <c r="Y18" s="33">
         <v>3</v>
       </c>
-      <c r="Z18" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="AA18" s="30" t="s">
+      <c r="Z18" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA18" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AB18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE18" s="29" t="s">
+      <c r="AB18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE18" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AF18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AG18" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH18" s="75"/>
-      <c r="AI18" s="27" t="s">
+      <c r="AF18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG18" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH18" s="74"/>
+      <c r="AI18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="AJ18" s="28">
+      <c r="AJ18" s="29">
         <v>6</v>
       </c>
-      <c r="AK18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL18" s="29" t="s">
+      <c r="AK18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL18" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AM18" s="30" t="s">
+      <c r="AM18" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AN18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AO18" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AP18" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AQ18" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AR18" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS18" s="79"/>
+      <c r="AN18" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO18" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AP18" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AQ18" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AR18" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS18" s="78"/>
     </row>
     <row r="19" ht="18.5" spans="1:45">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="32"/>
-      <c r="D19" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="E19" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="28" t="s">
+      <c r="C19" s="33"/>
+      <c r="D19" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="G19" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="H19" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I19" s="53" t="s">
+      <c r="G19" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="J19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="K19" s="51">
-        <v>40</v>
-      </c>
-      <c r="L19" s="52"/>
-      <c r="M19" s="27" t="s">
+      <c r="J19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="K19" s="50">
+        <v>40</v>
+      </c>
+      <c r="L19" s="51"/>
+      <c r="M19" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="N19" s="32">
+      <c r="N19" s="33">
         <v>3</v>
       </c>
-      <c r="O19" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="P19" s="30" t="s">
+      <c r="O19" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="P19" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="Q19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="R19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="S19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="T19" s="29" t="s">
+      <c r="Q19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="R19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="S19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="T19" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="U19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="V19" s="51">
-        <v>40</v>
-      </c>
-      <c r="W19" s="62"/>
-      <c r="X19" s="27" t="s">
+      <c r="U19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="V19" s="50">
+        <v>40</v>
+      </c>
+      <c r="W19" s="61"/>
+      <c r="X19" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="Y19" s="28">
+      <c r="Y19" s="29">
         <v>6</v>
       </c>
-      <c r="Z19" s="29" t="s">
+      <c r="Z19" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AA19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB19" s="30" t="s">
+      <c r="AA19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB19" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AC19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD19" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AE19" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AF19" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AG19" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH19" s="75"/>
-      <c r="AI19" s="27" t="s">
+      <c r="AC19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD19" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AE19" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF19" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AG19" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH19" s="74"/>
+      <c r="AI19" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="AJ19" s="32">
+      <c r="AJ19" s="33">
         <v>5</v>
       </c>
-      <c r="AK19" s="29" t="s">
+      <c r="AK19" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="AL19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AM19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AN19" s="29" t="s">
+      <c r="AL19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AM19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN19" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="AO19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AQ19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AR19" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS19" s="79"/>
+      <c r="AO19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AQ19" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AR19" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS19" s="78"/>
     </row>
     <row r="20" ht="18.5" spans="1:45">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="B20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="32">
+      <c r="C20" s="33">
         <v>3</v>
       </c>
-      <c r="D20" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" s="28" t="s">
+      <c r="D20" s="29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="F20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="H20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20" s="30" t="s">
+      <c r="F20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="J20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="K20" s="51">
-        <v>40</v>
-      </c>
-      <c r="L20" s="52"/>
-      <c r="M20" s="27" t="s">
+      <c r="J20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="K20" s="50">
+        <v>40</v>
+      </c>
+      <c r="L20" s="51"/>
+      <c r="M20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="N20" s="28">
+      <c r="N20" s="29">
         <v>6</v>
       </c>
-      <c r="O20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="P20" s="30" t="s">
+      <c r="O20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="P20" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="Q20" s="29" t="s">
+      <c r="Q20" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="R20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="S20" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="T20" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="U20" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="V20" s="51">
-        <v>40</v>
-      </c>
-      <c r="W20" s="62"/>
-      <c r="X20" s="27" t="s">
+      <c r="R20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="S20" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="T20" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="U20" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="V20" s="50">
+        <v>40</v>
+      </c>
+      <c r="W20" s="61"/>
+      <c r="X20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="Y20" s="32">
+      <c r="Y20" s="33">
         <v>5</v>
       </c>
-      <c r="Z20" s="29" t="s">
+      <c r="Z20" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="AA20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AB20" s="29" t="s">
+      <c r="AA20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB20" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="AC20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AE20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AF20" s="36" t="s">
+      <c r="AC20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE20" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF20" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="AG20" s="51">
-        <v>40</v>
-      </c>
-      <c r="AH20" s="52"/>
-      <c r="AI20" s="27" t="s">
+      <c r="AG20" s="50">
+        <v>40</v>
+      </c>
+      <c r="AH20" s="51"/>
+      <c r="AI20" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="AJ20" s="32"/>
-      <c r="AK20" s="36" t="s">
+      <c r="AJ20" s="33"/>
+      <c r="AK20" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AL20" s="36" t="s">
+      <c r="AL20" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AM20" s="36" t="s">
+      <c r="AM20" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AN20" s="36" t="s">
+      <c r="AN20" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="AO20" s="36" t="s">
+      <c r="AO20" s="37" t="s">
         <v>30</v>
       </c>
-      <c r="AP20" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AQ20" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="AR20" s="51">
-        <v>40</v>
-      </c>
-      <c r="AS20" s="80"/>
+      <c r="AP20" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AQ20" s="32" t="s">
+        <v>14</v>
+      </c>
+      <c r="AR20" s="50">
+        <v>40</v>
+      </c>
+      <c r="AS20" s="79"/>
     </row>
     <row r="21" ht="17.5" spans="1:45">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="28" t="s">
+      <c r="C21" s="11"/>
+      <c r="D21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="E21" s="28" t="s">
+      <c r="E21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="F21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="G21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="H21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I21" s="29" t="s">
+      <c r="F21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="G21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I21" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="K21" s="48"/>
-      <c r="L21" s="52"/>
-      <c r="M21" s="40" t="s">
+      <c r="K21" s="47"/>
+      <c r="L21" s="51"/>
+      <c r="M21" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="N21" s="9"/>
-      <c r="O21" s="28" t="s">
+      <c r="N21" s="11"/>
+      <c r="O21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="P21" s="28" t="s">
+      <c r="P21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="Q21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="R21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="S21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="T21" s="29" t="s">
+      <c r="Q21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="R21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="S21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="T21" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="U21" s="29" t="s">
+      <c r="U21" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="V21" s="48"/>
-      <c r="W21" s="62"/>
-      <c r="X21" s="40" t="s">
+      <c r="V21" s="47"/>
+      <c r="W21" s="61"/>
+      <c r="X21" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="Y21" s="9"/>
-      <c r="Z21" s="28" t="s">
+      <c r="Y21" s="11"/>
+      <c r="Z21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AA21" s="28" t="s">
+      <c r="AA21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AB21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AC21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD21" s="29" t="s">
+      <c r="AB21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD21" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="AE21" s="29" t="s">
+      <c r="AE21" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="AF21" s="29" t="s">
+      <c r="AF21" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="AG21" s="76"/>
-      <c r="AH21" s="52"/>
-      <c r="AI21" s="40" t="s">
+      <c r="AG21" s="75"/>
+      <c r="AH21" s="51"/>
+      <c r="AI21" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="AJ21" s="9"/>
-      <c r="AK21" s="28" t="s">
+      <c r="AJ21" s="11"/>
+      <c r="AK21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AL21" s="28" t="s">
+      <c r="AL21" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="AM21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AN21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AO21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP21" s="29" t="s">
+      <c r="AM21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AN21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO21" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP21" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="AQ21" s="29" t="s">
+      <c r="AQ21" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="AR21" s="76"/>
-      <c r="AS21" s="81"/>
+      <c r="AR21" s="75"/>
+      <c r="AS21" s="80"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4010,7 +4009,7 @@
     </row>
     <row r="3" ht="18.5" spans="1:2">
       <c r="A3" s="4" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B3" s="6">
         <v>46120</v>
@@ -4018,7 +4017,7 @@
     </row>
     <row r="4" ht="18.5" spans="1:2">
       <c r="A4" s="4" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B4" s="6">
         <v>46118</v>
@@ -4026,7 +4025,7 @@
     </row>
     <row r="5" ht="18.5" spans="1:2">
       <c r="A5" s="4" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="B5" s="6">
         <v>46121</v>
@@ -4034,7 +4033,7 @@
     </row>
     <row r="6" ht="18.5" spans="1:2">
       <c r="A6" s="4" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="B6" s="6">
         <v>46124</v>
@@ -4042,7 +4041,7 @@
     </row>
     <row r="7" ht="18.5" spans="1:2">
       <c r="A7" s="4" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="B7" s="6">
         <v>46123</v>
@@ -4050,7 +4049,7 @@
     </row>
     <row r="8" ht="18.5" spans="1:2">
       <c r="A8" s="4" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="B8" s="6">
         <v>46124</v>
@@ -4058,15 +4057,15 @@
     </row>
     <row r="9" ht="18.5" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="B9" s="6">
         <v>46121</v>
       </c>
     </row>
-    <row r="10" ht="18.5" spans="1:2">
-      <c r="A10" s="4" t="s">
-        <v>10</v>
+    <row r="10" ht="17.5" spans="1:2">
+      <c r="A10" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="B10" s="6">
         <v>46122</v>
@@ -4074,7 +4073,7 @@
     </row>
     <row r="11" ht="18.5" spans="1:2">
       <c r="A11" s="4" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="B11" s="6">
         <v>46122</v>
@@ -4082,7 +4081,7 @@
     </row>
     <row r="12" ht="18.5" spans="1:2">
       <c r="A12" s="4" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="B12" s="6">
         <v>46124</v>
@@ -4090,7 +4089,7 @@
     </row>
     <row r="13" ht="18.5" spans="1:2">
       <c r="A13" s="4" t="s">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B13" s="6">
         <v>46123</v>
@@ -4098,7 +4097,7 @@
     </row>
     <row r="14" ht="18.5" spans="1:2">
       <c r="A14" s="4" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="B14" s="6">
         <v>46120</v>
@@ -4106,7 +4105,7 @@
     </row>
     <row r="15" ht="18.5" spans="1:2">
       <c r="A15" s="4" t="s">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="B15" s="6">
         <v>46121</v>
@@ -4114,15 +4113,15 @@
     </row>
     <row r="16" ht="18.5" spans="1:2">
       <c r="A16" s="4" t="s">
-        <v>10</v>
+        <v>56</v>
       </c>
       <c r="B16" s="6">
         <v>46120</v>
       </c>
     </row>
-    <row r="17" ht="18.5" spans="1:2">
-      <c r="A17" s="4" t="s">
-        <v>10</v>
+    <row r="17" ht="17.5" spans="1:2">
+      <c r="A17" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="B17" s="6">
         <v>46124</v>

</xml_diff>